<commit_message>
feat: Update build cache and version information
- Updated file hashes in .build_cache.json to reflect recent changes.
- Added new assets and updated existing file paths to use forward slashes.
- Updated version.py to version 1.46.50 with new build date and version history.
- Modified build_unified.py to include additional source file patterns and adjusted hook paths.
- Enhanced verify_proc.ps1 to accept parameters for executable path and timeout, improving flexibility.
- Updated verify_gui.py to dynamically set project paths using pathlib.
- Updated various Excel files in test_config_sync and test_output directories.
</commit_message>
<xml_diff>
--- a/test_config_sync/source/test1.xlsx
+++ b/test_config_sync/source/test1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>